<commit_message>
Release v1.1.0 with email schedules, downtime reports and desktop builds
</commit_message>
<xml_diff>
--- a/templates/sitesentry_monitors_template.xlsx
+++ b/templates/sitesentry_monitors_template.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Monitors'!$A$1:$AB$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Monitors'!$A$1:$AD$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -61,7 +61,7 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB4"/>
+  <dimension ref="A1:AD4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -465,9 +465,11 @@
     <col width="18" customWidth="1" min="26" max="26"/>
     <col width="18" customWidth="1" min="27" max="27"/>
     <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="18" customWidth="1" min="30" max="30"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>id</t>
@@ -608,8 +610,18 @@
           <t>cooldown_minutes</t>
         </is>
       </c>
-    </row>
-    <row r="2">
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>web_server</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -676,8 +688,18 @@
       <c r="AB2" s="2" t="n">
         <v>30</v>
       </c>
-    </row>
-    <row r="3">
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>PHP</t>
+        </is>
+      </c>
+      <c r="AD2" s="2" t="inlineStr">
+        <is>
+          <t>Apache</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="2" t="inlineStr"/>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -756,8 +778,18 @@
       <c r="AB3" s="2" t="n">
         <v>30</v>
       </c>
-    </row>
-    <row r="4">
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="AD3" s="2" t="inlineStr">
+        <is>
+          <t>Nginx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="2" t="inlineStr"/>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -852,9 +884,19 @@
       <c r="AB4" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>ASP.NET</t>
+        </is>
+      </c>
+      <c r="AD4" s="2" t="inlineStr">
+        <is>
+          <t>IIS</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB1"/>
+  <autoFilter ref="A1:AD1"/>
   <dataValidations count="3">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"simple_web,auth_web,api"</formula1>
@@ -876,7 +918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -884,7 +926,7 @@
     <col width="100" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Column</t>
@@ -901,7 +943,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="34" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>id</t>
@@ -918,7 +960,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="34" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>name</t>
@@ -935,7 +977,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>monitor_type</t>
@@ -952,7 +994,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>enabled</t>
@@ -969,7 +1011,7 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="34" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>url</t>
@@ -986,88 +1028,122 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="34" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Application language/framework, for example PHP, Python, Java, ASP.NET.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>web_server</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Web server, for example Apache, Nginx, IIS, Tomcat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>headers_json</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>JSON object, for example {"Accept":"application/json"}.</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>body</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Request body for API methods such as POST/PUT/PATCH.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>api_token</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Stored encrypted after import.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>auth_password</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Stored encrypted after import.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>auth_extra_fields</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>JSON object with additional login form fields.</t>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>JSON object with additional login form fields. Hidden inputs are collected from the login page automatically.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: classify incidents before sending alerts
Add evidence-based diagnostics, per-monitor rules, network profiles, safer notification delivery and updated reports. Prepare the v1.3.0 release.
</commit_message>
<xml_diff>
--- a/templates/sitesentry_monitors_template.xlsx
+++ b/templates/sitesentry_monitors_template.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Monitors'!$A$1:$AD$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Monitors'!$A$1:$AF$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD4"/>
+  <dimension ref="A1:AF4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -467,6 +467,8 @@
     <col width="18" customWidth="1" min="28" max="28"/>
     <col width="18" customWidth="1" min="29" max="29"/>
     <col width="18" customWidth="1" min="30" max="30"/>
+    <col width="24" customWidth="1" min="31" max="31"/>
+    <col width="58" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -620,6 +622,16 @@
           <t>web_server</t>
         </is>
       </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>network_profile</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>diagnostic_rules_json</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr"/>
@@ -634,7 +646,7 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -698,8 +710,10 @@
           <t>Apache</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="42" customHeight="1">
+      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AF2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3" ht="84" customHeight="1">
       <c r="A3" s="2" t="inlineStr"/>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -712,7 +726,7 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
@@ -788,6 +802,12 @@
           <t>Nginx</t>
         </is>
       </c>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr">
+        <is>
+          <t>[{"id": "api-failure", "enabled": true, "priority": 100, "phase": "response", "conditions": [{"source": "json", "path": "success", "operator": "equals", "value": false}], "result": {"error_type": "assertion_failed", "reason_code": "business_rule_match"}}]</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="2" t="inlineStr"/>
@@ -894,9 +914,11 @@
           <t>IIS</t>
         </is>
       </c>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD1"/>
+  <autoFilter ref="A1:AF1"/>
   <dataValidations count="3">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"simple_web,auth_web,api"</formula1>
@@ -918,7 +940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1065,7 +1087,7 @@
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>headers_json</t>
+          <t>network_profile</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1075,14 +1097,14 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>JSON object, for example {"Accept":"application/json"}.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
+          <t>Existing network profile; blank preserves it; __CLEAR__ removes it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="56" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>body</t>
+          <t>diagnostic_rules_json</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1092,14 +1114,14 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Request body for API methods such as POST/PUT/PATCH.</t>
+          <t>JSON array of rules; blank preserves existing rules; [] clears them. See the Health API example and checker-spec.md §7. Configure profiles first.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="34" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>api_token</t>
+          <t>headers_json</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1109,14 +1131,14 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Stored encrypted after import.</t>
+          <t>JSON object, for example {"Accept":"application/json"}.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>auth_password</t>
+          <t>body</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1126,22 +1148,56 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Stored encrypted after import.</t>
+          <t>Request body for API methods such as POST/PUT/PATCH.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>api_token</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Stored encrypted after import.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>auth_password</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Stored encrypted after import.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>auth_extra_fields</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>JSON object with additional login form fields. Hidden inputs are collected from the login page automatically.</t>
         </is>

</xml_diff>